<commit_message>
feat: audit rules, reports, and dependency trace
</commit_message>
<xml_diff>
--- a/fixtures/clean_model.xlsx
+++ b/fixtures/clean_model.xlsx
@@ -615,8 +615,8 @@
         <v>21</v>
       </c>
       <c r="C3">
-        <f>Inputs!B2*0.1</f>
-        <v>100</v>
+        <f>Inputs!B2*Inputs!B3</f>
+        <v>30</v>
       </c>
       <c r="D3">
         <f>C3+1</f>

</xml_diff>